<commit_message>
Correct Bibliographie's suggested grade and break the 8b tie
Two curated patches, each cited in the module that carries it, and the
datasets and timeline figures rebuilt against them.

build_datasets.SUGGESTED_GRADE_PATCHES restores Megos's 9c proposal on
Bibliographie, which the scrape's structured field records as the 9b+ the
route settled at even though the prose on the same page describes the
downgrade. Every patch names the stale value it replaces and writes a
citation into suggested_grade_source, so a later scrape that fixes the
field upstream retires the correction instead of overwriting it silently.

milestones.TIE_BREAKS gives the first 8b to Kanal im Rücken, which carries
a real date, over Les Mains Sales, which is year-only and sorts first only
because a bare year anchors to 1 January. It applies only where the data
genuinely cannot order the pair, and the losing rival is still reported in
ordering_unresolved_with.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/processed/disputed_ascents.xlsx
+++ b/data/processed/disputed_ascents.xlsx
@@ -1147,13 +1147,13 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>9b+</t>
+          <t>9c</t>
         </is>
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr">
         <is>
-          <t>consensus</t>
+          <t>regraded</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -1179,7 +1179,7 @@
       </c>
       <c r="M11" t="inlineStr">
         <is>
-          <t>9b+</t>
+          <t>9c</t>
         </is>
       </c>
       <c r="N11" t="b">

</xml_diff>